<commit_message>
Water and nitrogen separated to DAHBSIM
</commit_message>
<xml_diff>
--- a/Dahbsim_PMP.xlsx
+++ b/Dahbsim_PMP.xlsx
@@ -413,16 +413,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>PMPsoln</t>
+        </is>
+      </c>
       <c r="D1" t="inlineStr">
-        <is>
-          <t>PMPsoln</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
         <is>
           <t>baseData</t>
         </is>
@@ -436,19 +436,14 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>barley_imp</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>field1</t>
-        </is>
+          <t>wheat_c</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>0.4299957</v>
       </c>
       <c r="D2" t="n">
-        <v>0.735642883730015</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0.536</v>
+        <v>0.43</v>
       </c>
     </row>
     <row r="3">
@@ -459,19 +454,14 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>barley_imp</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>field2</t>
-        </is>
+          <t>maize_c</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>0.2099978999999999</v>
       </c>
       <c r="D3" t="n">
-        <v>4.613258356365725e-13</v>
-      </c>
-      <c r="E3" t="n">
-        <v/>
+        <v>0.21</v>
       </c>
     </row>
     <row r="4">
@@ -482,18 +472,13 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>sorgum_imp</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>field1</t>
-        </is>
+          <t>imp_wheat</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>6.400000000094551e-06</v>
       </c>
       <c r="D4" t="n">
-        <v>-9.396558026787888e-11</v>
-      </c>
-      <c r="E4" t="n">
         <v/>
       </c>
     </row>
@@ -505,19 +490,14 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>sorgum_imp</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>field2</t>
-        </is>
+          <t>no_plant</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v/>
       </c>
       <c r="D5" t="n">
-        <v>6.683301182417875e-05</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0.258</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -528,410 +508,209 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>tomato_imp</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>field1</t>
+          <t>no_plant</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.3040000078581647</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0.28</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>hh_1</t>
+          <t>hh_2</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>tomato_imp</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>field2</t>
-        </is>
+          <t>clover_c</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0.1999979997891433</v>
       </c>
       <c r="D7" t="n">
-        <v>-9.709932896179317e-11</v>
-      </c>
-      <c r="E7" t="n">
-        <v/>
+        <v>0.2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>hh_1</t>
+          <t>hh_2</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>forage_imp</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>field1</t>
-        </is>
+          <t>sorghum_c</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0.1699983000973205</v>
       </c>
       <c r="D8" t="n">
-        <v>-9.395000431393029e-11</v>
-      </c>
-      <c r="E8" t="n">
-        <v/>
+        <v>0.17</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>hh_1</t>
+          <t>hh_2</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>forage_imp</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>field2</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>0.641000003582285</v>
-      </c>
-      <c r="E9" t="n">
-        <v>0.383</v>
+          <t>imp_wheat</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2.300210600485876e-06</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>hh_1</t>
+          <t>hh_2</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>oat_imp</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>field1</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>0.670357104877996</v>
-      </c>
-      <c r="E10" t="n">
-        <v>0.87</v>
+          <t>imp_wheat</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>9.29999999998987e-06</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>hh_1</t>
+          <t>hh_2</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>oat_imp</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>field2</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>1.399874289561098e-11</v>
-      </c>
-      <c r="E11" t="n">
-        <v/>
+          <t>imp_wheat</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1.067310982013983e-08</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>hh_1</t>
+          <t>hh_2</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>clover_imp</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>field1</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>2.657428054712245e-11</v>
-      </c>
-      <c r="E12" t="n">
-        <v/>
+          <t>imp_maize</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>6.04448298574796e-09</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>hh_1</t>
+          <t>hh_3</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>clover_imp</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>field2</t>
-        </is>
+          <t>wheat_c</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0.4499999503316934</v>
       </c>
       <c r="D13" t="n">
-        <v>0.3600000135174777</v>
-      </c>
-      <c r="E13" t="n">
-        <v>0.36</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>hh_1</t>
+          <t>hh_3</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>durumw_imp</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>field1</t>
-        </is>
+          <t>maize_c</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>0.3400000333766788</v>
       </c>
       <c r="D14" t="n">
-        <v>-9.392319256999175e-11</v>
-      </c>
-      <c r="E14" t="n">
-        <v/>
+        <v>0.34</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>hh_1</t>
+          <t>hh_3</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>durumw_imp</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>field2</t>
-        </is>
+          <t>clover_c</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>0.2183887902811951</v>
       </c>
       <c r="D15" t="n">
-        <v>0.05000000009874628</v>
-      </c>
-      <c r="E15" t="n">
-        <v>0.05</v>
+        <v>0.23</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>hh_1</t>
+          <t>hh_3</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>alfalfa_imp</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>field1</t>
-        </is>
+          <t>sorghum_c</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0.1116112102388093</v>
       </c>
       <c r="D16" t="n">
-        <v>-9.396802933470631e-11</v>
-      </c>
-      <c r="E16" t="n">
-        <v/>
+        <v>0.1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>hh_1</t>
+          <t>hh_3</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>alfalfa_imp</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>field2</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>0.05293314992300144</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0.053</v>
+          <t>imp_wheat</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>9.842530920484235e-09</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>hh_1</t>
+          <t>hh_3</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>petitpois_imp</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>field1</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>0.0180111494628579</v>
-      </c>
-      <c r="E18" t="n">
-        <v>0.016</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>hh_1</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>petitpois_imp</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>field2</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>1.966930499767512e-11</v>
-      </c>
-      <c r="E19" t="n">
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>hh_1</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>dolique_imp</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>field1</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>0.002988854521667041</v>
-      </c>
-      <c r="E20" t="n">
-        <v>0.021</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>hh_1</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>dolique_imp</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>field2</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>1.872560266322817e-11</v>
-      </c>
-      <c r="E21" t="n">
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>hh_1</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>chickpea_loc</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>field1</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>7.049701423291702e-11</v>
-      </c>
-      <c r="E22" t="n">
-        <v>0.008</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>hh_1</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>chickpea_loc</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>field2</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>2.036761094759173e-11</v>
-      </c>
-      <c r="E23" t="n">
-        <v/>
+          <t>imp_maize</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>5.946923437561556e-09</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Parameterization of biophysical module
Need some cleaning
</commit_message>
<xml_diff>
--- a/Dahbsim_PMP.xlsx
+++ b/Dahbsim_PMP.xlsx
@@ -413,16 +413,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>PMPsoln</t>
+        </is>
+      </c>
       <c r="D1" t="inlineStr">
-        <is>
-          <t>PMPsoln</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
         <is>
           <t>baseData</t>
         </is>
@@ -436,19 +436,14 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>barley_imp</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>field1</t>
-        </is>
+          <t>wheat_c</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>0.4299957</v>
       </c>
       <c r="D2" t="n">
-        <v>0.735642883730015</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0.536</v>
+        <v>0.43</v>
       </c>
     </row>
     <row r="3">
@@ -459,19 +454,14 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>barley_imp</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>field2</t>
-        </is>
+          <t>maize_c</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>0.2099978999999999</v>
       </c>
       <c r="D3" t="n">
-        <v>4.613258356365725e-13</v>
-      </c>
-      <c r="E3" t="n">
-        <v/>
+        <v>0.21</v>
       </c>
     </row>
     <row r="4">
@@ -482,18 +472,13 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>sorgum_imp</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>field1</t>
-        </is>
+          <t>imp_wheat</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>6.400000000094551e-06</v>
       </c>
       <c r="D4" t="n">
-        <v>-9.396558026787888e-11</v>
-      </c>
-      <c r="E4" t="n">
         <v/>
       </c>
     </row>
@@ -505,19 +490,14 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>sorgum_imp</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>field2</t>
-        </is>
+          <t>no_plant</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v/>
       </c>
       <c r="D5" t="n">
-        <v>6.683301182417875e-05</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0.258</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -528,410 +508,209 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>tomato_imp</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>field1</t>
+          <t>no_plant</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.3040000078581647</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0.28</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>hh_1</t>
+          <t>hh_2</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>tomato_imp</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>field2</t>
-        </is>
+          <t>clover_c</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0.1999979997891433</v>
       </c>
       <c r="D7" t="n">
-        <v>-9.709932896179317e-11</v>
-      </c>
-      <c r="E7" t="n">
-        <v/>
+        <v>0.2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>hh_1</t>
+          <t>hh_2</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>forage_imp</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>field1</t>
-        </is>
+          <t>sorghum_c</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0.1699983000973205</v>
       </c>
       <c r="D8" t="n">
-        <v>-9.395000431393029e-11</v>
-      </c>
-      <c r="E8" t="n">
-        <v/>
+        <v>0.17</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>hh_1</t>
+          <t>hh_2</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>forage_imp</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>field2</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>0.641000003582285</v>
-      </c>
-      <c r="E9" t="n">
-        <v>0.383</v>
+          <t>imp_wheat</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2.300210600485876e-06</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>hh_1</t>
+          <t>hh_2</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>oat_imp</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>field1</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>0.670357104877996</v>
-      </c>
-      <c r="E10" t="n">
-        <v>0.87</v>
+          <t>imp_wheat</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>9.29999999998987e-06</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>hh_1</t>
+          <t>hh_2</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>oat_imp</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>field2</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>1.399874289561098e-11</v>
-      </c>
-      <c r="E11" t="n">
-        <v/>
+          <t>imp_wheat</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1.067310982013983e-08</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>hh_1</t>
+          <t>hh_2</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>clover_imp</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>field1</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>2.657428054712245e-11</v>
-      </c>
-      <c r="E12" t="n">
-        <v/>
+          <t>imp_maize</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>6.04448298574796e-09</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>hh_1</t>
+          <t>hh_3</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>clover_imp</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>field2</t>
-        </is>
+          <t>wheat_c</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0.4499999503316934</v>
       </c>
       <c r="D13" t="n">
-        <v>0.3600000135174777</v>
-      </c>
-      <c r="E13" t="n">
-        <v>0.36</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>hh_1</t>
+          <t>hh_3</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>durumw_imp</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>field1</t>
-        </is>
+          <t>maize_c</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>0.3400000333766788</v>
       </c>
       <c r="D14" t="n">
-        <v>-9.392319256999175e-11</v>
-      </c>
-      <c r="E14" t="n">
-        <v/>
+        <v>0.34</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>hh_1</t>
+          <t>hh_3</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>durumw_imp</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>field2</t>
-        </is>
+          <t>clover_c</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>0.2183887902811951</v>
       </c>
       <c r="D15" t="n">
-        <v>0.05000000009874628</v>
-      </c>
-      <c r="E15" t="n">
-        <v>0.05</v>
+        <v>0.23</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>hh_1</t>
+          <t>hh_3</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>alfalfa_imp</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>field1</t>
-        </is>
+          <t>sorghum_c</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0.1116112102388093</v>
       </c>
       <c r="D16" t="n">
-        <v>-9.396802933470631e-11</v>
-      </c>
-      <c r="E16" t="n">
-        <v/>
+        <v>0.1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>hh_1</t>
+          <t>hh_3</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>alfalfa_imp</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>field2</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>0.05293314992300144</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0.053</v>
+          <t>imp_wheat</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>9.842530920484235e-09</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>hh_1</t>
+          <t>hh_3</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>petitpois_imp</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>field1</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>0.0180111494628579</v>
-      </c>
-      <c r="E18" t="n">
-        <v>0.016</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>hh_1</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>petitpois_imp</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>field2</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>1.966930499767512e-11</v>
-      </c>
-      <c r="E19" t="n">
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>hh_1</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>dolique_imp</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>field1</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>0.002988854521667041</v>
-      </c>
-      <c r="E20" t="n">
-        <v>0.021</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>hh_1</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>dolique_imp</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>field2</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>1.872560266322817e-11</v>
-      </c>
-      <c r="E21" t="n">
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>hh_1</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>chickpea_loc</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>field1</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>7.049701423291702e-11</v>
-      </c>
-      <c r="E22" t="n">
-        <v>0.008</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>hh_1</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>chickpea_loc</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>field2</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>2.036761094759173e-11</v>
-      </c>
-      <c r="E23" t="n">
-        <v/>
+          <t>imp_maize</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>5.946923437561556e-09</v>
       </c>
     </row>
   </sheetData>

</xml_diff>